<commit_message>
Add budget cycles core: Cycles ledger, /cycle command, salary prompt, cycle-scoped summary and budget
</commit_message>
<xml_diff>
--- a/data/Expenses_Template.xlsx
+++ b/data/Expenses_Template.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="📖 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MasterData" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Monthly Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📖 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MasterData" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cycles" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1210,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A2:F54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="114" min="1" max="1"/>
@@ -16490,4 +16491,30 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>StartDate</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: rename Value/Budget (PLN) columns to (base)
</commit_message>
<xml_diff>
--- a/data/Expenses_Template.xlsx
+++ b/data/Expenses_Template.xlsx
@@ -1211,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F54"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="114" min="1" max="1"/>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="D1" s="0" t="inlineStr">
         <is>
-          <t>Budget (PLN)</t>
+          <t>Budget (base)</t>
         </is>
       </c>
       <c r="E1" s="39" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="L1" s="40" t="inlineStr">
         <is>
-          <t>Value (PLN)</t>
+          <t>Value (base)</t>
         </is>
       </c>
     </row>
@@ -14442,6 +14442,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="114">
       <c r="A4" s="90" t="inlineStr">
         <is>
@@ -14512,6 +14513,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="19.5" customHeight="1" s="114">
       <c r="A9" s="90" t="inlineStr">
         <is>
@@ -16503,12 +16505,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>StartDate</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>Label</t>
         </is>

</xml_diff>

<commit_message>
fix: complete _pln->_base rename, sync template header, add workbook migration script
</commit_message>
<xml_diff>
--- a/data/Expenses_Template.xlsx
+++ b/data/Expenses_Template.xlsx
@@ -1211,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A2:F54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="114" min="1" max="1"/>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="I1" s="40" t="inlineStr">
         <is>
-          <t>Rate to PLN</t>
+          <t>Rate to base</t>
         </is>
       </c>
       <c r="M1" s="123" t="inlineStr">
@@ -14442,7 +14442,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="114">
       <c r="A4" s="90" t="inlineStr">
         <is>
@@ -14513,7 +14512,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="19.5" customHeight="1" s="114">
       <c r="A9" s="90" t="inlineStr">
         <is>

</xml_diff>